<commit_message>
v0.2.0: sections-driven rendering, scaffold/render mode split, exported typst_escape/cv_section/resolve_date_fun, why-curriculr vignette
</commit_message>
<xml_diff>
--- a/inst/extdata/cv-data-template.xlsx
+++ b/inst/extdata/cv-data-template.xlsx
@@ -5,34 +5,35 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lares/Documents/projects/curriculr/ins/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lares/Documents/projects/curriculr/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EADFEFED-41AA-784E-9FC6-4787B77DD32A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51955D10-5BA1-A744-B1BE-ED31788ABB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6220" yWindow="600" windowWidth="70580" windowHeight="31400" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33120" yWindow="3980" windowWidth="41940" windowHeight="23260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile" sheetId="1" r:id="rId1"/>
-    <sheet name="education" sheetId="2" r:id="rId2"/>
-    <sheet name="experience" sheetId="3" r:id="rId3"/>
-    <sheet name="projects" sheetId="4" r:id="rId4"/>
-    <sheet name="publications" sheetId="5" r:id="rId5"/>
-    <sheet name="presentations" sheetId="6" r:id="rId6"/>
-    <sheet name="invited_teaching" sheetId="7" r:id="rId7"/>
-    <sheet name="grants_and_awards" sheetId="8" r:id="rId8"/>
-    <sheet name="certifications" sheetId="9" r:id="rId9"/>
-    <sheet name="admin_services" sheetId="10" r:id="rId10"/>
-    <sheet name="skills" sheetId="11" r:id="rId11"/>
-    <sheet name="affiliations" sheetId="12" r:id="rId12"/>
-    <sheet name="readme" sheetId="13" r:id="rId13"/>
+    <sheet name="sections" sheetId="14" r:id="rId2"/>
+    <sheet name="education" sheetId="2" r:id="rId3"/>
+    <sheet name="experience" sheetId="3" r:id="rId4"/>
+    <sheet name="projects" sheetId="4" r:id="rId5"/>
+    <sheet name="publications" sheetId="5" r:id="rId6"/>
+    <sheet name="presentations" sheetId="6" r:id="rId7"/>
+    <sheet name="invited_teaching" sheetId="7" r:id="rId8"/>
+    <sheet name="grants_and_awards" sheetId="8" r:id="rId9"/>
+    <sheet name="certifications" sheetId="9" r:id="rId10"/>
+    <sheet name="admin_services" sheetId="10" r:id="rId11"/>
+    <sheet name="skills" sheetId="11" r:id="rId12"/>
+    <sheet name="affiliations" sheetId="12" r:id="rId13"/>
+    <sheet name="readme" sheetId="15" r:id="rId14"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="269">
   <si>
     <t>field</t>
   </si>
@@ -493,9 +494,6 @@
     <t>Relative path to your profile image, e.g.  img/me-profile.png</t>
   </si>
   <si>
-    <t>One or two sentence professional summary shown below the contact line</t>
-  </si>
-  <si>
     <t>LinkedIn path, e.g.  in/erwin-lares  (no URL prefix)</t>
   </si>
   <si>
@@ -520,12 +518,6 @@
     <t>Your first name, displayed in the CV header</t>
   </si>
   <si>
-    <t>What it controls</t>
-  </si>
-  <si>
-    <t>Profile Tab Reference</t>
-  </si>
-  <si>
     <t>(leave blank)</t>
   </si>
   <si>
@@ -535,9 +527,6 @@
     <t>2023</t>
   </si>
   <si>
-    <t>Single month/year event (presentation)</t>
-  </si>
-  <si>
     <t>2021</t>
   </si>
   <si>
@@ -574,21 +563,9 @@
     <t>Situation</t>
   </si>
   <si>
-    <t>Date Entry Quick Reference</t>
-  </si>
-  <si>
-    <t>Never — always enter TRUE or FALSE for these sheets</t>
-  </si>
-  <si>
-    <t>TRUE or FALSE. Controls whether this entry appears in a short resume variant.</t>
-  </si>
-  <si>
     <t>education, experience</t>
   </si>
   <si>
-    <t>Never — always classify your publications</t>
-  </si>
-  <si>
     <t>One of:  book  |  essay  |  periodical  |  interview  |  chapter</t>
   </si>
   <si>
@@ -598,100 +575,293 @@
     <t>No further detail is needed</t>
   </si>
   <si>
-    <t>A one- or two-sentence description, institutional affiliation, or additional context.</t>
-  </si>
-  <si>
     <t>most sheets</t>
   </si>
   <si>
     <t>Location is not relevant or not known</t>
   </si>
   <si>
-    <t>City and state or country, e.g.  Madison, WI  or  London, UK</t>
-  </si>
-  <si>
-    <t>The role is ongoing (pair with  present  in endMonth), or the entry is a point-in-time event</t>
-  </si>
-  <si>
     <t>Four-digit year.</t>
   </si>
   <si>
     <t>dated sheets</t>
   </si>
   <si>
-    <t>The entry is a point-in-time event such as an award or publication — leave both endMonth and endYear blank</t>
-  </si>
-  <si>
-    <t>Three-letter abbreviation (Dec), OR the word  present  if the role is ongoing.</t>
-  </si>
-  <si>
-    <t>The section does not use dates (skills, affiliations)</t>
-  </si>
-  <si>
     <t>Four-digit year, e.g. 2019</t>
   </si>
   <si>
-    <t>You only want year-level precision, or the section does not use dates (skills, affiliations)</t>
-  </si>
-  <si>
-    <t>Three-letter month abbreviation: Jan, Feb, Mar, Apr, May, Jun, Jul, Aug, Sep, Oct, Nov, Dec</t>
-  </si>
-  <si>
-    <t>Never — required for all education entries</t>
-  </si>
-  <si>
     <t>The degree-granting institution.</t>
   </si>
   <si>
     <t>education only</t>
   </si>
   <si>
-    <t>No secondary organization applies to this entry</t>
-  </si>
-  <si>
-    <t>The secondary organization, employer, publisher, or venue associated with the entry.</t>
-  </si>
-  <si>
-    <t>Never — this column is always required</t>
-  </si>
-  <si>
-    <t>The primary label for the entry: degree name, job title, project name, skill area, publication title, etc.</t>
-  </si>
-  <si>
     <t>all sheets</t>
   </si>
   <si>
-    <t>Leave blank when</t>
-  </si>
-  <si>
-    <t>What to enter</t>
-  </si>
-  <si>
-    <t>Applies to</t>
-  </si>
-  <si>
-    <t>Column</t>
-  </si>
-  <si>
-    <t>Column Reference</t>
+    <t>curriculr Workbook Guide</t>
+  </si>
+  <si>
+    <t>No date rendered</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>Single year: "2021"</t>
+  </si>
+  <si>
+    <t>year_only</t>
+  </si>
+  <si>
+    <t>Single point in time: "Jan 2018"</t>
+  </si>
+  <si>
+    <t>month_year</t>
+  </si>
+  <si>
+    <t>Year range only: "2018 - 2022" or "2018"</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>Full month/year range: "Jan 2018 - Dec 2022" or "Jan 2018 - Present"</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>what it produces</t>
+  </si>
+  <si>
+    <t>token</t>
+  </si>
+  <si>
+    <t>date_fun token reference</t>
+  </si>
+  <si>
+    <t>Affiliations</t>
+  </si>
+  <si>
+    <t>affiliations</t>
+  </si>
+  <si>
+    <t>Skills</t>
+  </si>
+  <si>
+    <t>skills</t>
+  </si>
+  <si>
+    <t>Administrative Services</t>
+  </si>
+  <si>
+    <t>admin_services</t>
+  </si>
+  <si>
+    <t>Grants and Awards</t>
+  </si>
+  <si>
+    <t>grants_and_awards</t>
+  </si>
+  <si>
+    <t>Certifications</t>
+  </si>
+  <si>
+    <t>certifications</t>
+  </si>
+  <si>
+    <t>Presentations</t>
+  </si>
+  <si>
+    <t>presentations</t>
+  </si>
+  <si>
+    <t>Publications</t>
+  </si>
+  <si>
+    <t>publications</t>
+  </si>
+  <si>
+    <t>Invited Teaching</t>
+  </si>
+  <si>
+    <t>invited_teaching</t>
+  </si>
+  <si>
+    <t>Projects</t>
+  </si>
+  <si>
+    <t>projects</t>
+  </si>
+  <si>
+    <t>Experience</t>
+  </si>
+  <si>
+    <t>experience</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>education</t>
+  </si>
+  <si>
+    <t>where_col</t>
+  </si>
+  <si>
+    <t>date_fun</t>
+  </si>
+  <si>
+    <t>detail_col</t>
+  </si>
+  <si>
+    <t>org_col</t>
+  </si>
+  <si>
+    <t>title_col</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>section</t>
   </si>
   <si>
     <t>This workbook is the single source of truth for your CV. Each tab corresponds to one section of the CV. Edit the data in the appropriate tab and re-render CV.qmd to update your PDF.
 • Do not add, remove, or rename columns — column names are read by R and must match exactly.
 • You can add as many rows as you need within any tab.
-• Leave a cell blank (do not type NA) when a value does not apply to an entry.</t>
-  </si>
-  <si>
-    <t>curriculr Workbook Guide</t>
+• Leave a cell blank (do not type NA) when a value does not apply to an entry.
+• The sections tab controls which sections appear in the CV and in what order.
+• To exclude a section, delete its row from the sections tab.
+• To reorder sections, reorder the rows in the sections tab.</t>
+  </si>
+  <si>
+    <t>The sections tab</t>
+  </si>
+  <si>
+    <t>The sections tab controls which CV sections are rendered and in what order. Each row corresponds to one section. The order of rows is the order of sections in the PDF. To remove a section from the CV, delete its row. To add a new section, add a new row — as long as the section name matches a sheet in this workbook and the sheet follows the standard column schema, it will render automatically.</t>
+  </si>
+  <si>
+    <t>sections tab columns</t>
+  </si>
+  <si>
+    <t>column</t>
+  </si>
+  <si>
+    <t>what it controls</t>
+  </si>
+  <si>
+    <t>Must match a sheet name exactly, e.g. education, grants_and_awards</t>
+  </si>
+  <si>
+    <t>The section heading displayed in the rendered PDF, e.g. "Grants &amp; Awards"</t>
+  </si>
+  <si>
+    <t>Column used as the primary entry label</t>
+  </si>
+  <si>
+    <t>Column used as the secondary organization or venue line. Leave blank to omit.</t>
+  </si>
+  <si>
+    <t>Column used as the detail or description line. Leave blank to omit.</t>
+  </si>
+  <si>
+    <t>Token controlling date formatting. See date_fun reference below.</t>
+  </si>
+  <si>
+    <t>Column used as the location. Leave blank to omit.</t>
+  </si>
+  <si>
+    <t>date_fun tokens</t>
+  </si>
+  <si>
+    <t>Column reference — section data tabs</t>
+  </si>
+  <si>
+    <t>applies to</t>
+  </si>
+  <si>
+    <t>what to enter</t>
+  </si>
+  <si>
+    <t>leave blank when</t>
+  </si>
+  <si>
+    <t>The primary label for the entry: degree name, job title, project name, skill area, etc.</t>
+  </si>
+  <si>
+    <t>Never — always required</t>
+  </si>
+  <si>
+    <t>The secondary organization, employer, publisher, or venue.</t>
+  </si>
+  <si>
+    <t>No secondary organization applies</t>
+  </si>
+  <si>
+    <t>Never — required for education entries</t>
+  </si>
+  <si>
+    <t>Three-letter abbreviation: Jan, Feb, Mar, Apr, May, Jun, Jul, Aug, Sep, Oct, Nov, Dec</t>
+  </si>
+  <si>
+    <t>You only want year-level precision, or the section does not use dates</t>
+  </si>
+  <si>
+    <t>The section does not use dates</t>
+  </si>
+  <si>
+    <t>Three-letter abbreviation, OR the word  present  if the role is ongoing.</t>
+  </si>
+  <si>
+    <t>The entry is a point-in-time event — leave both endMonth and endYear blank</t>
+  </si>
+  <si>
+    <t>The role is ongoing (pair with  present  in endMonth), or a point-in-time event</t>
+  </si>
+  <si>
+    <t>City and state or country, e.g.  Madison, WI</t>
+  </si>
+  <si>
+    <t>A one- or two-sentence description or additional context.</t>
+  </si>
+  <si>
+    <t>Never — always classify publications</t>
+  </si>
+  <si>
+    <t>TRUE or FALSE. Reserved for future resume variant support.</t>
+  </si>
+  <si>
+    <t>Never — always enter TRUE or FALSE</t>
+  </si>
+  <si>
+    <t>Date entry quick reference</t>
+  </si>
+  <si>
+    <t>Single month/year (presentation)</t>
+  </si>
+  <si>
+    <t>Profile tab reference</t>
+  </si>
+  <si>
+    <t>One or two sentence professional summary</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -712,26 +882,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF303030"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF303030"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFC5050C"/>
@@ -748,6 +898,31 @@
     <font>
       <b/>
       <sz val="14"/>
+      <color rgb="FFC5050C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color rgb="FFC5050C"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -795,59 +970,62 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{AC82B805-010D-CF46-9C40-7812B59A1EAE}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{791263E9-A613-6B46-8713-827121E9760F}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1249,6 +1427,75 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="10" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3">
+        <v>2020</v>
+      </c>
+      <c r="G3" t="s">
+        <v>111</v>
+      </c>
+      <c r="H3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1361,7 +1608,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1434,7 +1681,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1474,456 +1721,923 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A6C21C-7AA1-A048-BCDA-4352462E3285}">
-  <dimension ref="A1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBB777-E3A1-AF4C-B7CC-8F0FC5346FEE}">
+  <dimension ref="A1:E68"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18" style="2" customWidth="1"/>
-    <col min="2" max="2" width="22" style="2" customWidth="1"/>
+    <col min="1" max="2" width="22" style="2" customWidth="1"/>
     <col min="3" max="3" width="52" style="2" customWidth="1"/>
     <col min="4" max="4" width="42" style="2" customWidth="1"/>
-    <col min="5" max="5" width="20" style="2" customWidth="1"/>
+    <col min="5" max="5" width="16" style="2" customWidth="1"/>
     <col min="6" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
-        <v>215</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-    </row>
-    <row r="2" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
+      <c r="A1" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+    </row>
+    <row r="2" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
     </row>
     <row r="3" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+    <row r="4" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+    </row>
+    <row r="6" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="7" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="8" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="B27" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B28" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="8" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D43" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="D44" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="B46" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E46" s="15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="8" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="8" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="39" x14ac:dyDescent="0.2">
+      <c r="A64" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="26" x14ac:dyDescent="0.2">
+      <c r="A65" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="26" x14ac:dyDescent="0.2">
+      <c r="A66" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B68" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="8" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>152</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A5:D5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B35A59F4-434E-4C48-B517-A4C3874BEB43}">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24" style="2" customWidth="1"/>
+    <col min="2" max="2" width="28" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14" style="2" customWidth="1"/>
+    <col min="4" max="4" width="16" style="2" customWidth="1"/>
+    <col min="5" max="6" width="14" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="G11" s="5"/>
+    </row>
+    <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G12" s="3"/>
+    </row>
+    <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="17" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="20" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2007,7 +2721,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2135,7 +2849,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2254,7 +2968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2381,7 +3095,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2522,7 +3236,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2623,7 +3337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2744,73 +3458,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="10" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D2">
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B3" t="s">
-        <v>110</v>
-      </c>
-      <c r="D3">
-        <v>2020</v>
-      </c>
-      <c r="G3" t="s">
-        <v>111</v>
-      </c>
-      <c r="H3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
v0.3.0: resume variant, Font Awesome icons, theming, add_section()
</commit_message>
<xml_diff>
--- a/inst/extdata/cv-data-template.xlsx
+++ b/inst/extdata/cv-data-template.xlsx
@@ -8,32 +8,105 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lares/Documents/projects/curriculr/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51955D10-5BA1-A744-B1BE-ED31788ABB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{566332D5-A048-7B46-B265-C813BEBBA649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33120" yWindow="3980" windowWidth="41940" windowHeight="23260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14660" yWindow="3980" windowWidth="60400" windowHeight="24520" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile" sheetId="1" r:id="rId1"/>
-    <sheet name="sections" sheetId="14" r:id="rId2"/>
-    <sheet name="education" sheetId="2" r:id="rId3"/>
-    <sheet name="experience" sheetId="3" r:id="rId4"/>
-    <sheet name="projects" sheetId="4" r:id="rId5"/>
-    <sheet name="publications" sheetId="5" r:id="rId6"/>
-    <sheet name="presentations" sheetId="6" r:id="rId7"/>
-    <sheet name="invited_teaching" sheetId="7" r:id="rId8"/>
-    <sheet name="grants_and_awards" sheetId="8" r:id="rId9"/>
-    <sheet name="certifications" sheetId="9" r:id="rId10"/>
-    <sheet name="admin_services" sheetId="10" r:id="rId11"/>
-    <sheet name="skills" sheetId="11" r:id="rId12"/>
-    <sheet name="affiliations" sheetId="12" r:id="rId13"/>
-    <sheet name="readme" sheetId="15" r:id="rId14"/>
+    <sheet name="sections" sheetId="2" r:id="rId2"/>
+    <sheet name="education" sheetId="3" r:id="rId3"/>
+    <sheet name="experience" sheetId="4" r:id="rId4"/>
+    <sheet name="projects" sheetId="5" r:id="rId5"/>
+    <sheet name="publications" sheetId="6" r:id="rId6"/>
+    <sheet name="presentations" sheetId="7" r:id="rId7"/>
+    <sheet name="invited_teaching" sheetId="8" r:id="rId8"/>
+    <sheet name="grants_and_awards" sheetId="9" r:id="rId9"/>
+    <sheet name="certifications" sheetId="10" r:id="rId10"/>
+    <sheet name="admin_services" sheetId="11" r:id="rId11"/>
+    <sheet name="skills" sheetId="12" r:id="rId12"/>
+    <sheet name="affiliations" sheetId="13" r:id="rId13"/>
+    <sheet name="theme" sheetId="14" r:id="rId14"/>
+    <sheet name="readme" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="322">
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>startMonth</t>
+  </si>
+  <si>
+    <t>startYear</t>
+  </si>
+  <si>
+    <t>endMonth</t>
+  </si>
+  <si>
+    <t>endYear</t>
+  </si>
+  <si>
+    <t>where</t>
+  </si>
+  <si>
+    <t>detail</t>
+  </si>
+  <si>
+    <t>include_in_resume</t>
+  </si>
+  <si>
+    <t>Master Class: Ink and Watercolor Technique</t>
+  </si>
+  <si>
+    <t>Society of Illustrators</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>New York, NY</t>
+  </si>
+  <si>
+    <t>One-day intensive for working illustrators. 24 participants.</t>
+  </si>
+  <si>
+    <t>Editorial Illustration Workshop</t>
+  </si>
+  <si>
+    <t>Sequential Artists Workshop</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Gainesville, FL</t>
+  </si>
+  <si>
+    <t>Three-day workshop. Focus on ideation under deadline.</t>
+  </si>
+  <si>
+    <t>Character Design Intensive</t>
+  </si>
+  <si>
+    <t>Illustration Academy</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Kansas City, MO</t>
+  </si>
+  <si>
+    <t>Week-long summer intensive for advanced illustration students.</t>
+  </si>
   <si>
     <t>field</t>
   </si>
@@ -101,25 +174,109 @@
     <t>img/frank-profile.png</t>
   </si>
   <si>
-    <t>title</t>
-  </si>
-  <si>
-    <t>startYear</t>
-  </si>
-  <si>
-    <t>endYear</t>
+    <t>section</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>title_col</t>
+  </si>
+  <si>
+    <t>org_col</t>
+  </si>
+  <si>
+    <t>detail_col</t>
+  </si>
+  <si>
+    <t>date_fun</t>
+  </si>
+  <si>
+    <t>where_col</t>
+  </si>
+  <si>
+    <t>education</t>
+  </si>
+  <si>
+    <t>Education</t>
   </si>
   <si>
     <t>institution</t>
   </si>
   <si>
-    <t>where</t>
-  </si>
-  <si>
-    <t>detail</t>
-  </si>
-  <si>
-    <t>include_in_resume</t>
+    <t>year</t>
+  </si>
+  <si>
+    <t>experience</t>
+  </si>
+  <si>
+    <t>Experience</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>projects</t>
+  </si>
+  <si>
+    <t>Projects</t>
+  </si>
+  <si>
+    <t>invited_teaching</t>
+  </si>
+  <si>
+    <t>Invited Teaching</t>
+  </si>
+  <si>
+    <t>month_year</t>
+  </si>
+  <si>
+    <t>publications</t>
+  </si>
+  <si>
+    <t>Publications</t>
+  </si>
+  <si>
+    <t>year_only</t>
+  </si>
+  <si>
+    <t>presentations</t>
+  </si>
+  <si>
+    <t>Presentations</t>
+  </si>
+  <si>
+    <t>certifications</t>
+  </si>
+  <si>
+    <t>Certifications</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>grants_and_awards</t>
+  </si>
+  <si>
+    <t>Grants and Awards</t>
+  </si>
+  <si>
+    <t>admin_services</t>
+  </si>
+  <si>
+    <t>Administrative Services</t>
+  </si>
+  <si>
+    <t>skills</t>
+  </si>
+  <si>
+    <t>Skills</t>
+  </si>
+  <si>
+    <t>affiliations</t>
+  </si>
+  <si>
+    <t>Affiliations</t>
   </si>
   <si>
     <t>Bachelor of Fine Arts, Illustration</t>
@@ -146,15 +303,6 @@
     <t>Competitive residency program. Studied under noted figurative painters.</t>
   </si>
   <si>
-    <t>unit</t>
-  </si>
-  <si>
-    <t>startMonth</t>
-  </si>
-  <si>
-    <t>endMonth</t>
-  </si>
-  <si>
     <t>Principal Illustrator</t>
   </si>
   <si>
@@ -179,9 +327,6 @@
     <t>The Portland Tribune</t>
   </si>
   <si>
-    <t>Mar</t>
-  </si>
-  <si>
     <t>Dec</t>
   </si>
   <si>
@@ -221,9 +366,6 @@
     <t>Oregon Mycological Society</t>
   </si>
   <si>
-    <t>Jun</t>
-  </si>
-  <si>
     <t>Apr</t>
   </si>
   <si>
@@ -236,9 +378,6 @@
     <t>Regional Arts &amp; Culture Council</t>
   </si>
   <si>
-    <t>Aug</t>
-  </si>
-  <si>
     <t>60-foot exterior mural commissioned for the Central Eastside Arts District. Depicted the city's history of migration and trade.</t>
   </si>
   <si>
@@ -278,9 +417,6 @@
     <t>The New Yorker</t>
   </si>
   <si>
-    <t>New York, NY</t>
-  </si>
-  <si>
     <t>periodical</t>
   </si>
   <si>
@@ -353,39 +489,6 @@
     <t>Workshop facilitator.</t>
   </si>
   <si>
-    <t>Master Class: Ink and Watercolor Technique</t>
-  </si>
-  <si>
-    <t>Society of Illustrators</t>
-  </si>
-  <si>
-    <t>One-day intensive for working illustrators. 24 participants.</t>
-  </si>
-  <si>
-    <t>Editorial Illustration Workshop</t>
-  </si>
-  <si>
-    <t>Sequential Artists Workshop</t>
-  </si>
-  <si>
-    <t>Gainesville, FL</t>
-  </si>
-  <si>
-    <t>Three-day workshop. Focus on ideation under deadline.</t>
-  </si>
-  <si>
-    <t>Character Design Intensive</t>
-  </si>
-  <si>
-    <t>Illustration Academy</t>
-  </si>
-  <si>
-    <t>Kansas City, MO</t>
-  </si>
-  <si>
-    <t>Week-long summer intensive for advanced illustration students.</t>
-  </si>
-  <si>
     <t>Eisner Award Shortlist, Best Graphic Album—New</t>
   </si>
   <si>
@@ -491,241 +594,121 @@
     <t>Authors Guild</t>
   </si>
   <si>
-    <t>Relative path to your profile image, e.g.  img/me-profile.png</t>
-  </si>
-  <si>
-    <t>LinkedIn path, e.g.  in/erwin-lares  (no URL prefix)</t>
-  </si>
-  <si>
-    <t>GitHub username only, e.g.  erwinlares  (no URL prefix)</t>
-  </si>
-  <si>
-    <t>Personal or professional website URL</t>
-  </si>
-  <si>
-    <t>Email address — the @ will be escaped automatically</t>
-  </si>
-  <si>
-    <t>Mailing address shown in the contact line</t>
-  </si>
-  <si>
-    <t>Your current title or professional identity line</t>
-  </si>
-  <si>
-    <t>Your last name, displayed in the CV header</t>
-  </si>
-  <si>
-    <t>Your first name, displayed in the CV header</t>
-  </si>
-  <si>
-    <t>(leave blank)</t>
-  </si>
-  <si>
-    <t>No date (skills, affiliations)</t>
-  </si>
-  <si>
-    <t>2023</t>
-  </si>
-  <si>
-    <t>2021</t>
-  </si>
-  <si>
-    <t>Single-year event (award, publication)</t>
-  </si>
-  <si>
-    <t>2014</t>
-  </si>
-  <si>
-    <t>2010</t>
-  </si>
-  <si>
-    <t>Completed role — year only</t>
-  </si>
-  <si>
-    <t>2018</t>
-  </si>
-  <si>
-    <t>Ongoing role — year only</t>
-  </si>
-  <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>2015</t>
-  </si>
-  <si>
-    <t>Completed role — month precision</t>
-  </si>
-  <si>
-    <t>Ongoing role — month precision</t>
-  </si>
-  <si>
-    <t>Situation</t>
-  </si>
-  <si>
-    <t>education, experience</t>
-  </si>
-  <si>
-    <t>One of:  book  |  essay  |  periodical  |  interview  |  chapter</t>
-  </si>
-  <si>
-    <t>publications only</t>
-  </si>
-  <si>
-    <t>No further detail is needed</t>
-  </si>
-  <si>
-    <t>most sheets</t>
-  </si>
-  <si>
-    <t>Location is not relevant or not known</t>
-  </si>
-  <si>
-    <t>Four-digit year.</t>
-  </si>
-  <si>
-    <t>dated sheets</t>
-  </si>
-  <si>
-    <t>Four-digit year, e.g. 2019</t>
-  </si>
-  <si>
-    <t>The degree-granting institution.</t>
-  </si>
-  <si>
-    <t>education only</t>
-  </si>
-  <si>
-    <t>all sheets</t>
+    <t>key</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>font_family</t>
+  </si>
+  <si>
+    <t>Lato</t>
+  </si>
+  <si>
+    <t>Body font. Must be available to Typst.</t>
+  </si>
+  <si>
+    <t>font_size</t>
+  </si>
+  <si>
+    <t>8.8pt</t>
+  </si>
+  <si>
+    <t>Base font size for body text.</t>
+  </si>
+  <si>
+    <t>body_color</t>
+  </si>
+  <si>
+    <t>#3f3f3f</t>
+  </si>
+  <si>
+    <t>Main body text color.</t>
+  </si>
+  <si>
+    <t>line_leading</t>
+  </si>
+  <si>
+    <t>0.48em</t>
+  </si>
+  <si>
+    <t>Spacing between lines of text.</t>
+  </si>
+  <si>
+    <t>accent_color</t>
+  </si>
+  <si>
+    <t>#c5050c</t>
+  </si>
+  <si>
+    <t>Section headings, dates, and ruled lines accent.</t>
+  </si>
+  <si>
+    <t>dark_color</t>
+  </si>
+  <si>
+    <t>#303030</t>
+  </si>
+  <si>
+    <t>Entry titles and name in the header.</t>
+  </si>
+  <si>
+    <t>bodygray_color</t>
+  </si>
+  <si>
+    <t>#555555</t>
+  </si>
+  <si>
+    <t>Organization and detail lines.</t>
+  </si>
+  <si>
+    <t>lightgray_color</t>
+  </si>
+  <si>
+    <t>#777777</t>
+  </si>
+  <si>
+    <t>Address and contact line.</t>
+  </si>
+  <si>
+    <t>rulegray_color</t>
+  </si>
+  <si>
+    <t>#d9d9d9</t>
+  </si>
+  <si>
+    <t>Horizontal rule under section headings.</t>
+  </si>
+  <si>
+    <t>papersize</t>
+  </si>
+  <si>
+    <t>us-letter</t>
+  </si>
+  <si>
+    <t>Page size. Common values: us-letter, a4.</t>
+  </si>
+  <si>
+    <t>margin_x</t>
+  </si>
+  <si>
+    <t>0.62in</t>
+  </si>
+  <si>
+    <t>Left and right page margins.</t>
+  </si>
+  <si>
+    <t>margin_y</t>
+  </si>
+  <si>
+    <t>0.58in</t>
+  </si>
+  <si>
+    <t>Top and bottom page margins.</t>
   </si>
   <si>
     <t>curriculr Workbook Guide</t>
-  </si>
-  <si>
-    <t>No date rendered</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>Single year: "2021"</t>
-  </si>
-  <si>
-    <t>year_only</t>
-  </si>
-  <si>
-    <t>Single point in time: "Jan 2018"</t>
-  </si>
-  <si>
-    <t>month_year</t>
-  </si>
-  <si>
-    <t>Year range only: "2018 - 2022" or "2018"</t>
-  </si>
-  <si>
-    <t>year</t>
-  </si>
-  <si>
-    <t>Full month/year range: "Jan 2018 - Dec 2022" or "Jan 2018 - Present"</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>what it produces</t>
-  </si>
-  <si>
-    <t>token</t>
-  </si>
-  <si>
-    <t>date_fun token reference</t>
-  </si>
-  <si>
-    <t>Affiliations</t>
-  </si>
-  <si>
-    <t>affiliations</t>
-  </si>
-  <si>
-    <t>Skills</t>
-  </si>
-  <si>
-    <t>skills</t>
-  </si>
-  <si>
-    <t>Administrative Services</t>
-  </si>
-  <si>
-    <t>admin_services</t>
-  </si>
-  <si>
-    <t>Grants and Awards</t>
-  </si>
-  <si>
-    <t>grants_and_awards</t>
-  </si>
-  <si>
-    <t>Certifications</t>
-  </si>
-  <si>
-    <t>certifications</t>
-  </si>
-  <si>
-    <t>Presentations</t>
-  </si>
-  <si>
-    <t>presentations</t>
-  </si>
-  <si>
-    <t>Publications</t>
-  </si>
-  <si>
-    <t>publications</t>
-  </si>
-  <si>
-    <t>Invited Teaching</t>
-  </si>
-  <si>
-    <t>invited_teaching</t>
-  </si>
-  <si>
-    <t>Projects</t>
-  </si>
-  <si>
-    <t>projects</t>
-  </si>
-  <si>
-    <t>Experience</t>
-  </si>
-  <si>
-    <t>experience</t>
-  </si>
-  <si>
-    <t>Education</t>
-  </si>
-  <si>
-    <t>education</t>
-  </si>
-  <si>
-    <t>where_col</t>
-  </si>
-  <si>
-    <t>date_fun</t>
-  </si>
-  <si>
-    <t>detail_col</t>
-  </si>
-  <si>
-    <t>org_col</t>
-  </si>
-  <si>
-    <t>title_col</t>
-  </si>
-  <si>
-    <t>label</t>
-  </si>
-  <si>
-    <t>section</t>
   </si>
   <si>
     <t>This workbook is the single source of truth for your CV. Each tab corresponds to one section of the CV. Edit the data in the appropriate tab and re-render CV.qmd to update your PDF.
@@ -776,6 +759,27 @@
     <t>date_fun tokens</t>
   </si>
   <si>
+    <t>token</t>
+  </si>
+  <si>
+    <t>what it produces</t>
+  </si>
+  <si>
+    <t>Full month/year range: "Jan 2018 - Dec 2022" or "Jan 2018 - Present"</t>
+  </si>
+  <si>
+    <t>Year range only: "2018 - 2022" or "2018"</t>
+  </si>
+  <si>
+    <t>Single point in time: "Jan 2018"</t>
+  </si>
+  <si>
+    <t>Single year: "2021"</t>
+  </si>
+  <si>
+    <t>No date rendered</t>
+  </si>
+  <si>
     <t>Column reference — section data tabs</t>
   </si>
   <si>
@@ -788,27 +792,45 @@
     <t>leave blank when</t>
   </si>
   <si>
+    <t>all sheets</t>
+  </si>
+  <si>
     <t>The primary label for the entry: degree name, job title, project name, skill area, etc.</t>
   </si>
   <si>
     <t>Never — always required</t>
   </si>
   <si>
+    <t>most sheets</t>
+  </si>
+  <si>
     <t>The secondary organization, employer, publisher, or venue.</t>
   </si>
   <si>
     <t>No secondary organization applies</t>
   </si>
   <si>
+    <t>education only</t>
+  </si>
+  <si>
+    <t>The degree-granting institution.</t>
+  </si>
+  <si>
     <t>Never — required for education entries</t>
   </si>
   <si>
+    <t>dated sheets</t>
+  </si>
+  <si>
     <t>Three-letter abbreviation: Jan, Feb, Mar, Apr, May, Jun, Jul, Aug, Sep, Oct, Nov, Dec</t>
   </si>
   <si>
     <t>You only want year-level precision, or the section does not use dates</t>
   </si>
   <si>
+    <t>Four-digit year, e.g. 2019</t>
+  </si>
+  <si>
     <t>The section does not use dates</t>
   </si>
   <si>
@@ -818,18 +840,36 @@
     <t>The entry is a point-in-time event — leave both endMonth and endYear blank</t>
   </si>
   <si>
+    <t>Four-digit year.</t>
+  </si>
+  <si>
     <t>The role is ongoing (pair with  present  in endMonth), or a point-in-time event</t>
   </si>
   <si>
     <t>City and state or country, e.g.  Madison, WI</t>
   </si>
   <si>
+    <t>Location is not relevant or not known</t>
+  </si>
+  <si>
     <t>A one- or two-sentence description or additional context.</t>
   </si>
   <si>
+    <t>No further detail is needed</t>
+  </si>
+  <si>
+    <t>publications only</t>
+  </si>
+  <si>
+    <t>One of:  book  |  essay  |  periodical  |  interview  |  chapter</t>
+  </si>
+  <si>
     <t>Never — always classify publications</t>
   </si>
   <si>
+    <t>all section sheets</t>
+  </si>
+  <si>
     <t>TRUE or FALSE. Reserved for future resume variant support.</t>
   </si>
   <si>
@@ -839,20 +879,140 @@
     <t>Date entry quick reference</t>
   </si>
   <si>
+    <t>Situation</t>
+  </si>
+  <si>
+    <t>Ongoing role — month precision</t>
+  </si>
+  <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>(leave blank)</t>
+  </si>
+  <si>
+    <t>Completed role — month precision</t>
+  </si>
+  <si>
+    <t>2015</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>Ongoing role — year only</t>
+  </si>
+  <si>
+    <t>Completed role — year only</t>
+  </si>
+  <si>
+    <t>2010</t>
+  </si>
+  <si>
+    <t>2014</t>
+  </si>
+  <si>
+    <t>Single-year event (award, publication)</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
     <t>Single month/year (presentation)</t>
   </si>
   <si>
+    <t>2023</t>
+  </si>
+  <si>
+    <t>No date (skills, affiliations)</t>
+  </si>
+  <si>
     <t>Profile tab reference</t>
   </si>
   <si>
+    <t>Your first name, displayed in the CV header</t>
+  </si>
+  <si>
+    <t>Your last name, displayed in the CV header</t>
+  </si>
+  <si>
+    <t>Your current title or professional identity line</t>
+  </si>
+  <si>
+    <t>Mailing address shown in the contact line</t>
+  </si>
+  <si>
+    <t>Email address — the @ will be escaped automatically</t>
+  </si>
+  <si>
+    <t>Personal or professional website URL</t>
+  </si>
+  <si>
+    <t>GitHub username only, e.g.  erwinlares  (no URL prefix)</t>
+  </si>
+  <si>
+    <t>LinkedIn path, e.g.  in/erwin-lares  (no URL prefix)</t>
+  </si>
+  <si>
     <t>One or two sentence professional summary</t>
+  </si>
+  <si>
+    <t>Relative path to your profile image, e.g.  img/me-profile.png</t>
+  </si>
+  <si>
+    <t>date_fun token reference</t>
+  </si>
+  <si>
+    <t>Theme tab reference</t>
+  </si>
+  <si>
+    <t>The theme tab controls the visual appearance of the rendered CV. Edit the value column to change fonts, colors, and page layout. The description column is documentation only — changes to it have no effect.</t>
+  </si>
+  <si>
+    <t>value / what it controls</t>
+  </si>
+  <si>
+    <t>Body font name. Must be available to Typst, e.g. Lato, Arial, Times New Roman.</t>
+  </si>
+  <si>
+    <t>Base font size for body text, e.g. 8.8pt, 9pt, 10pt.</t>
+  </si>
+  <si>
+    <t>Main body text color. Hex code, e.g. #3f3f3f.</t>
+  </si>
+  <si>
+    <t>Line spacing. Smaller values tighten text, e.g. 0.48em.</t>
+  </si>
+  <si>
+    <t>Color used for section headings, dates, and rules. Hex code.</t>
+  </si>
+  <si>
+    <t>Color used for entry titles and the name in the header. Hex code.</t>
+  </si>
+  <si>
+    <t>Color used for organization and detail lines. Hex code.</t>
+  </si>
+  <si>
+    <t>Color used for address and contact line. Hex code.</t>
+  </si>
+  <si>
+    <t>Color of the horizontal rule under section headings. Hex code.</t>
+  </si>
+  <si>
+    <t>Page size. Use us-letter for North America, a4 for Europe.</t>
+  </si>
+  <si>
+    <t>Left and right page margins, e.g. 0.62in, 1.5cm.</t>
+  </si>
+  <si>
+    <t>Top and bottom page margins, e.g. 0.58in, 1.5cm.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -927,8 +1087,51 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF777777"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -939,6 +1142,19 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC5050C"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAF0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC5050C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -975,7 +1191,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
@@ -1014,6 +1230,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1021,11 +1245,25 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{AC82B805-010D-CF46-9C40-7812B59A1EAE}"/>
-    <cellStyle name="Normal 3" xfId="2" xr:uid="{791263E9-A613-6B46-8713-827121E9760F}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1038,6 +1276,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1335,90 +1590,90 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1427,8 +1682,8 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1436,58 +1691,67 @@
     <col min="3" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
       <c r="D2">
         <v>2022</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>133</v>
+        <v>167</v>
       </c>
       <c r="B3" t="s">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="D3">
         <v>2020</v>
       </c>
       <c r="G3" t="s">
-        <v>111</v>
+        <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>134</v>
+        <v>168</v>
+      </c>
+      <c r="I3" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1496,8 +1760,8 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:H4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1505,102 +1769,114 @@
     <col min="3" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>2022</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="F2">
         <v>2022</v>
       </c>
       <c r="G2" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="H2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>170</v>
+      </c>
+      <c r="I2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>171</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>2015</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="F3">
         <v>2019</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+      <c r="I3" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>139</v>
+        <v>173</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>2012</v>
       </c>
       <c r="E4" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="H4" t="s">
-        <v>140</v>
+        <v>174</v>
+      </c>
+      <c r="I4" s="27" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1609,8 +1885,8 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:H5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1618,62 +1894,77 @@
     <col min="3" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>141</v>
+        <v>175</v>
       </c>
       <c r="B2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+      <c r="I2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>143</v>
+        <v>177</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>178</v>
+      </c>
+      <c r="I3" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>179</v>
       </c>
       <c r="B4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>180</v>
+      </c>
+      <c r="I4" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>181</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>182</v>
+      </c>
+      <c r="I5" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1682,8 +1973,8 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:A5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1691,29 +1982,44 @@
     <col min="3" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="B2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+        <v>183</v>
+      </c>
+      <c r="B3" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+        <v>184</v>
+      </c>
+      <c r="B4" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>185</v>
+      </c>
+      <c r="B5" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1722,631 +2028,903 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBB777-E3A1-AF4C-B7CC-8F0FC5346FEE}">
-  <dimension ref="A1:E68"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="52" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>219</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>223</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="22" style="2" customWidth="1"/>
     <col min="3" max="3" width="52" style="2" customWidth="1"/>
     <col min="4" max="4" width="42" style="2" customWidth="1"/>
     <col min="5" max="5" width="16" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="8.83203125" style="2"/>
+    <col min="6" max="6" width="8.83203125" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="A1" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
     </row>
     <row r="2" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
+      <c r="A2" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
+      <c r="A5" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>230</v>
+        <v>46</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>229</v>
+        <v>47</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>228</v>
+        <v>48</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>227</v>
+        <v>49</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>226</v>
+        <v>50</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>225</v>
+        <v>51</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>224</v>
+        <v>52</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>200</v>
+        <v>239</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>199</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>197</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
-        <v>196</v>
+        <v>56</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>195</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>194</v>
+        <v>64</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>193</v>
+        <v>243</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
-        <v>192</v>
+        <v>67</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>191</v>
+        <v>244</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>189</v>
+        <v>245</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>187</v>
+        <v>250</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>180</v>
+        <v>253</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>186</v>
+        <v>256</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>185</v>
+        <v>257</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>184</v>
+        <v>262</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>182</v>
+        <v>266</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>180</v>
+        <v>253</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>181</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>180</v>
+        <v>253</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>179</v>
+        <v>271</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>178</v>
+        <v>272</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>177</v>
+        <v>273</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>176</v>
+        <v>275</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>175</v>
+        <v>279</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="10" t="s">
-        <v>174</v>
+        <v>280</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>169</v>
+        <v>281</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13" t="s">
-        <v>173</v>
+        <v>283</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>172</v>
+        <v>284</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>171</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="10" t="s">
-        <v>170</v>
+        <v>286</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>169</v>
+        <v>281</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13" t="s">
-        <v>168</v>
+        <v>287</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>167</v>
+        <v>288</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>166</v>
+        <v>289</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10" t="s">
-        <v>165</v>
+        <v>290</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>164</v>
+        <v>291</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13" t="s">
-        <v>266</v>
+        <v>292</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>90</v>
+        <v>135</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>163</v>
+        <v>293</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10" t="s">
-        <v>162</v>
+        <v>294</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>161</v>
+        <v>282</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="8" t="s">
-        <v>267</v>
+        <v>295</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>160</v>
+        <v>296</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>159</v>
+        <v>297</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>158</v>
+        <v>298</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>157</v>
+        <v>299</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>156</v>
+        <v>300</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>155</v>
+        <v>301</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>302</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>153</v>
+        <v>303</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>268</v>
+        <v>304</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>152</v>
+        <v>305</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="8" t="s">
-        <v>201</v>
+        <v>306</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>200</v>
+        <v>239</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="39" x14ac:dyDescent="0.2">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="26" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
-        <v>196</v>
+        <v>56</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="26" x14ac:dyDescent="0.2">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>194</v>
+        <v>64</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>193</v>
+        <v>243</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
-        <v>192</v>
+        <v>67</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>191</v>
+        <v>244</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>189</v>
+        <v>245</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="19" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="20" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="B73" s="21" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="B74" s="22" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="B75" s="23" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="B76" s="22" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="B77" s="23" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="B78" s="22" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="B79" s="23" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="B80" s="22" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B81" s="23" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="B82" s="22" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" s="23" t="s">
+        <v>215</v>
+      </c>
+      <c r="B83" s="23" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" s="22" t="s">
+        <v>218</v>
+      </c>
+      <c r="B84" s="22" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="B85" s="23" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -2360,7 +2938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B35A59F4-434E-4C48-B517-A4C3874BEB43}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2370,258 +2948,259 @@
     <col min="4" max="4" width="16" style="2" customWidth="1"/>
     <col min="5" max="6" width="14" style="2" customWidth="1"/>
     <col min="7" max="7" width="12" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.83203125" style="2"/>
+    <col min="8" max="8" width="8.83203125" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>230</v>
+        <v>46</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>229</v>
+        <v>47</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>228</v>
+        <v>48</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>227</v>
+        <v>49</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>226</v>
+        <v>50</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>225</v>
+        <v>51</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>224</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>223</v>
+        <v>53</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>222</v>
+        <v>54</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>196</v>
+        <v>56</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>221</v>
+        <v>57</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>220</v>
+        <v>58</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>219</v>
+        <v>60</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>218</v>
+        <v>61</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>217</v>
+        <v>62</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>216</v>
+        <v>63</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
-        <v>194</v>
+        <v>64</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>215</v>
+        <v>65</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>214</v>
+        <v>66</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>192</v>
+        <v>67</v>
       </c>
       <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>213</v>
+        <v>68</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>212</v>
+        <v>69</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>194</v>
+        <v>64</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>211</v>
+        <v>70</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>210</v>
+        <v>71</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="G8" s="3"/>
     </row>
     <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>209</v>
+        <v>73</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>208</v>
+        <v>74</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>207</v>
+        <v>75</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>206</v>
+        <v>76</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>205</v>
+        <v>77</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>204</v>
+        <v>78</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>203</v>
+        <v>79</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>202</v>
+        <v>80</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="G12" s="3"/>
     </row>
@@ -2638,7 +3217,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2649,30 +3228,30 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
+      </c>
+      <c r="G1" s="28" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="B2">
         <v>1990</v>
@@ -2681,21 +3260,21 @@
         <v>1994</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>82</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="F2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" t="b">
+        <v>84</v>
+      </c>
+      <c r="G2" s="27" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="B3">
         <v>1993</v>
@@ -2704,15 +3283,15 @@
         <v>1993</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" t="b">
+        <v>88</v>
+      </c>
+      <c r="G3" s="27" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2722,7 +3301,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2733,114 +3312,114 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
+      </c>
+      <c r="I1" s="28" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>1997</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I2" t="b">
+        <v>94</v>
+      </c>
+      <c r="I2" s="27" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="D3">
         <v>1994</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="F3">
         <v>1996</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I3" t="b">
+        <v>98</v>
+      </c>
+      <c r="I3" s="27" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>101</v>
       </c>
       <c r="D4">
         <v>2005</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="F4">
         <v>2014</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
-      </c>
-      <c r="I4" t="b">
+        <v>103</v>
+      </c>
+      <c r="I4" s="27" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2850,127 +3429,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="10" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2">
-        <v>2020</v>
-      </c>
-      <c r="E2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2">
-        <v>2022</v>
-      </c>
-      <c r="G2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3">
-        <v>2018</v>
-      </c>
-      <c r="E3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F3">
-        <v>2019</v>
-      </c>
-      <c r="G3" t="s">
-        <v>44</v>
-      </c>
-      <c r="H3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4">
-        <v>2016</v>
-      </c>
-      <c r="E4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4">
-        <v>2016</v>
-      </c>
-      <c r="G4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2980,114 +3440,118 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>105</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
       </c>
       <c r="D2">
+        <v>2020</v>
+      </c>
+      <c r="E2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2">
         <v>2022</v>
       </c>
       <c r="G2" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
-      </c>
-      <c r="I2" t="s">
-        <v>74</v>
+        <v>107</v>
+      </c>
+      <c r="I2" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="D3">
+        <v>2018</v>
+      </c>
+      <c r="E3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F3">
         <v>2019</v>
       </c>
+      <c r="G3" t="s">
+        <v>93</v>
+      </c>
       <c r="H3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I3" t="s">
-        <v>78</v>
+        <v>111</v>
+      </c>
+      <c r="I3" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>112</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>102</v>
       </c>
       <c r="D4">
-        <v>2015</v>
+        <v>2016</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4">
+        <v>2016</v>
       </c>
       <c r="G4" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="H4" t="s">
-        <v>82</v>
-      </c>
-      <c r="I4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5">
-        <v>2010</v>
-      </c>
-      <c r="H5" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" t="s">
-        <v>87</v>
+        <v>114</v>
+      </c>
+      <c r="I4" s="27" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3095,9 +3559,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3105,130 +3569,131 @@
     <col min="3" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C2" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
       <c r="D2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G2" t="s">
-        <v>81</v>
+        <v>118</v>
       </c>
       <c r="H2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3">
+        <v>2019</v>
+      </c>
+      <c r="H3" t="s">
+        <v>123</v>
+      </c>
+      <c r="I3" t="s">
+        <v>124</v>
+      </c>
+      <c r="J3" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>2015</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>127</v>
+      </c>
+      <c r="I4" t="s">
+        <v>128</v>
+      </c>
+      <c r="J4" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D3">
-        <v>2021</v>
-      </c>
-      <c r="G3" t="s">
-        <v>95</v>
-      </c>
-      <c r="H3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4">
-        <v>2018</v>
-      </c>
-      <c r="G4" t="s">
-        <v>81</v>
-      </c>
-      <c r="H4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" t="s">
-        <v>63</v>
-      </c>
       <c r="D5">
-        <v>2017</v>
-      </c>
-      <c r="G5" t="s">
-        <v>44</v>
+        <v>2010</v>
       </c>
       <c r="H5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6">
-        <v>2012</v>
-      </c>
-      <c r="G6" t="s">
-        <v>104</v>
-      </c>
-      <c r="H6" t="s">
-        <v>105</v>
+        <v>131</v>
+      </c>
+      <c r="I5" t="s">
+        <v>132</v>
+      </c>
+      <c r="J5" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3236,9 +3701,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3246,90 +3711,148 @@
     <col min="3" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+      <c r="I1" s="28" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2">
+        <v>2023</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>136</v>
+      </c>
+      <c r="I2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3">
+        <v>2021</v>
+      </c>
+      <c r="G3" t="s">
+        <v>140</v>
+      </c>
+      <c r="H3" t="s">
+        <v>141</v>
+      </c>
+      <c r="I3" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" t="s">
         <v>106</v>
       </c>
-      <c r="B2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2">
-        <v>2022</v>
-      </c>
-      <c r="G2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D4">
+        <v>2018</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I4" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" t="s">
         <v>110</v>
       </c>
-      <c r="C3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3">
-        <v>2019</v>
-      </c>
-      <c r="G3" t="s">
-        <v>111</v>
-      </c>
-      <c r="H3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4">
-        <v>2016</v>
-      </c>
-      <c r="G4" t="s">
-        <v>115</v>
-      </c>
-      <c r="H4" t="s">
-        <v>116</v>
+      <c r="D5">
+        <v>2017</v>
+      </c>
+      <c r="G5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I5" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>2012</v>
+      </c>
+      <c r="G6" t="s">
+        <v>149</v>
+      </c>
+      <c r="H6" t="s">
+        <v>150</v>
+      </c>
+      <c r="I6" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3337,9 +3860,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3347,112 +3870,243 @@
     <col min="3" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2">
+        <v>2022</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3">
+        <v>2019</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4">
+        <v>2016</v>
+      </c>
+      <c r="G4" t="s">
         <v>22</v>
       </c>
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="10" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+      <c r="I1" s="28" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="D2">
         <v>2023</v>
       </c>
       <c r="G2" t="s">
-        <v>119</v>
+        <v>153</v>
       </c>
       <c r="H2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>154</v>
+      </c>
+      <c r="I2" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="D3">
         <v>2021</v>
       </c>
       <c r="G3" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="H3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>156</v>
+      </c>
+      <c r="I3" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
+        <v>158</v>
       </c>
       <c r="D4">
         <v>2017</v>
       </c>
       <c r="G4" t="s">
-        <v>104</v>
+        <v>149</v>
       </c>
       <c r="H4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+      <c r="I4" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <v>2014</v>
       </c>
       <c r="G5" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="H5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+      <c r="I5" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>128</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
       <c r="D6">
         <v>2009</v>
       </c>
       <c r="H6" t="s">
-        <v>130</v>
+        <v>164</v>
+      </c>
+      <c r="I6" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>